<commit_message>
added code for figures
</commit_message>
<xml_diff>
--- a/data/evidence_factor_search_records.xlsx
+++ b/data/evidence_factor_search_records.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\My Drive\work\Projects\In_progress\conservation_evidence_factors_synthesis\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\work\Projects\In_progress\conservation_evidence_factors_synthesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B014A8F-9EEE-4575-B1DF-0EB632A4218F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36725F33-81C1-4880-996D-ACEA4F88B89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="9225" activeTab="2" xr2:uid="{6E12F9A6-757F-44E9-B59F-62645BD9B3E3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6E12F9A6-757F-44E9-B59F-62645BD9B3E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark studies" sheetId="2" r:id="rId1"/>
@@ -22,6 +22,20 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -290,24 +304,6 @@
     <t>Excluded full texts (not in English)</t>
   </si>
   <si>
-    <t>Excluded full texts (no population)</t>
-  </si>
-  <si>
-    <t>Excluded full texts (no biodiversity outcome)</t>
-  </si>
-  <si>
-    <t>Excluded full texts (no exposure)</t>
-  </si>
-  <si>
-    <t>Excluded full texts (not field based)</t>
-  </si>
-  <si>
-    <t>Excluded full texts (no comparison)</t>
-  </si>
-  <si>
-    <t>Excluded full texts (no PECO element)</t>
-  </si>
-  <si>
     <t>Total excluded texts at full-text</t>
   </si>
   <si>
@@ -330,6 +326,24 @@
   </si>
   <si>
     <t>Articles removed by automation</t>
+  </si>
+  <si>
+    <t>Excluded full texts (not a primary study)</t>
+  </si>
+  <si>
+    <t>Excluded full texts (wrong study design)</t>
+  </si>
+  <si>
+    <t>Excluded full texts (no about conservation)</t>
+  </si>
+  <si>
+    <t>Excluded full texts (not about policy or practice)</t>
+  </si>
+  <si>
+    <t>Excluded full texts (not about evidence use)</t>
+  </si>
+  <si>
+    <t>Excluded full texts (not about factors influencing evidence use)</t>
   </si>
 </sst>
 </file>
@@ -415,9 +429,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -455,7 +469,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -561,7 +575,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -703,7 +717,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1686,22 +1700,22 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72DD040-8C1B-456C-B7AE-50AD8B46E076}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>77</v>
       </c>
@@ -1709,15 +1723,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B3">
         <v>37938</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -1725,106 +1739,115 @@
         <v>8353</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B5" s="4">
-        <v>13087</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>13907</v>
+      </c>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>78</v>
       </c>
       <c r="B6" s="5">
         <f>B3-(B4+B5)</f>
-        <v>16498</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15678</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B8" s="5">
+        <f>B6-B7</f>
+        <v>15033</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version submitted to Journal of Applied Ecology in January 2025
</commit_message>
<xml_diff>
--- a/data/evidence_factor_search_records.xlsx
+++ b/data/evidence_factor_search_records.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\work\Projects\In_progress\conservation_evidence_factors_synthesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36725F33-81C1-4880-996D-ACEA4F88B89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC38C26-765B-4532-A030-C84062848150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6E12F9A6-757F-44E9-B59F-62645BD9B3E3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6E12F9A6-757F-44E9-B59F-62645BD9B3E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark studies" sheetId="2" r:id="rId1"/>
@@ -334,9 +334,6 @@
     <t>Excluded full texts (wrong study design)</t>
   </si>
   <si>
-    <t>Excluded full texts (no about conservation)</t>
-  </si>
-  <si>
     <t>Excluded full texts (not about policy or practice)</t>
   </si>
   <si>
@@ -344,6 +341,9 @@
   </si>
   <si>
     <t>Excluded full texts (not about factors influencing evidence use)</t>
+  </si>
+  <si>
+    <t>Excluded full texts (not about conservation)</t>
   </si>
 </sst>
 </file>
@@ -1695,6 +1695,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1754,8 +1755,12 @@
         <v>78</v>
       </c>
       <c r="B6" s="5">
-        <f>B3-(B4+B5)</f>
-        <v>15678</v>
+        <f>B3-(B4)</f>
+        <v>29585</v>
+      </c>
+      <c r="D6" s="5">
+        <f>B6-13087</f>
+        <v>16498</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1763,7 +1768,7 @@
         <v>80</v>
       </c>
       <c r="B7">
-        <v>645</v>
+        <v>736</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1772,82 +1777,134 @@
       </c>
       <c r="B8" s="5">
         <f>B6-B7</f>
-        <v>15033</v>
+        <v>28849</v>
+      </c>
+      <c r="D8" s="5">
+        <f>B8-13087</f>
+        <v>15762</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>82</v>
       </c>
+      <c r="B9">
+        <f>B7-(B10+B11)</f>
+        <v>726</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>83</v>
       </c>
+      <c r="B10">
+        <v>6</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>84</v>
       </c>
+      <c r="B11">
+        <v>4</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>85</v>
       </c>
+      <c r="B12">
+        <v>167</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>86</v>
       </c>
+      <c r="B13">
+        <v>4</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>95</v>
       </c>
+      <c r="B14">
+        <v>282</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
+      <c r="B15">
+        <v>70</v>
+      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B18">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <f>SUM(B13:B19)</f>
+        <v>549</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <f>B9-(B10+B11+B20)</f>
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>90</v>
+      </c>
+      <c r="B23">
+        <v>167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cleaning up folders for archiving
</commit_message>
<xml_diff>
--- a/data/evidence_factor_search_records.xlsx
+++ b/data/evidence_factor_search_records.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\work\Projects\In_progress\conservation_evidence_factors_synthesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DC38C26-765B-4532-A030-C84062848150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732D5A70-E631-408D-A18A-04EF70084CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6E12F9A6-757F-44E9-B59F-62645BD9B3E3}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6E12F9A6-757F-44E9-B59F-62645BD9B3E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark studies" sheetId="2" r:id="rId1"/>
@@ -1758,10 +1758,7 @@
         <f>B3-(B4)</f>
         <v>29585</v>
       </c>
-      <c r="D6" s="5">
-        <f>B6-13087</f>
-        <v>16498</v>
-      </c>
+      <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">

</xml_diff>

<commit_message>
tidying up files for archiving
</commit_message>
<xml_diff>
--- a/data/evidence_factor_search_records.xlsx
+++ b/data/evidence_factor_search_records.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\work\Projects\In_progress\conservation_evidence_factors_synthesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{732D5A70-E631-408D-A18A-04EF70084CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0DED933-D4E8-48F0-BB05-251B1FDE4102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6E12F9A6-757F-44E9-B59F-62645BD9B3E3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{6E12F9A6-757F-44E9-B59F-62645BD9B3E3}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark studies" sheetId="2" r:id="rId1"/>
@@ -726,14 +726,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68DA44D2-0179-4F11-B929-311EC031542E}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="4.42578125" customWidth="1"/>
-    <col min="2" max="2" width="114.140625" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
+    <col min="1" max="1" width="4.453125" customWidth="1"/>
+    <col min="2" max="2" width="114.1796875" customWidth="1"/>
+    <col min="4" max="4" width="16.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -750,7 +750,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -767,7 +767,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -784,7 +784,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -801,7 +801,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -818,7 +818,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -835,7 +835,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -852,7 +852,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -869,7 +869,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -886,7 +886,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -903,7 +903,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -941,13 +941,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFEB4CD3-B81D-4935-A650-7301C27E6529}">
   <dimension ref="A1:AB13"/>
-  <sheetFormatPr defaultColWidth="34.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="34.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="135.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="135.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1013,7 +1013,7 @@
       <c r="AA1" s="1"/>
       <c r="AB1" s="1"/>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1181,7 +1181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1238,7 +1238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1295,7 +1295,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1352,7 +1352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>10</v>
       </c>
@@ -1523,7 +1523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>11</v>
       </c>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>12</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>13</v>
       </c>
@@ -1702,13 +1702,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72DD040-8C1B-456C-B7AE-50AD8B46E076}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="41.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="41.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>91</v>
       </c>
@@ -1716,7 +1716,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>77</v>
       </c>
@@ -1724,7 +1724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>93</v>
       </c>
@@ -1732,7 +1732,7 @@
         <v>37938</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -1740,7 +1740,7 @@
         <v>8353</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -1750,7 +1750,7 @@
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>78</v>
       </c>
@@ -1758,17 +1758,24 @@
         <f>B3-(B4)</f>
         <v>29585</v>
       </c>
-      <c r="D6" s="5"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="5">
+        <f>B6-B5</f>
+        <v>15678</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>80</v>
       </c>
       <c r="B7">
         <v>736</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="5">
+        <f>D6-B7</f>
+        <v>14942</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>81</v>
       </c>
@@ -1781,7 +1788,7 @@
         <v>15762</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>82</v>
       </c>
@@ -1790,7 +1797,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>83</v>
       </c>
@@ -1798,7 +1805,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>84</v>
       </c>
@@ -1806,7 +1813,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -1814,7 +1821,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>86</v>
       </c>
@@ -1822,7 +1829,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>95</v>
       </c>
@@ -1830,7 +1837,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -1838,7 +1845,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>100</v>
       </c>
@@ -1846,7 +1853,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>97</v>
       </c>
@@ -1854,7 +1861,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>98</v>
       </c>
@@ -1862,7 +1869,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>99</v>
       </c>
@@ -1870,7 +1877,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>87</v>
       </c>
@@ -1879,7 +1886,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>88</v>
       </c>
@@ -1888,7 +1895,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>89</v>
       </c>
@@ -1896,7 +1903,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>90</v>
       </c>

</xml_diff>